<commit_message>
Actualización 28 Feb: Nuevo formato pagado_pendiente, ajustes en Legión Centurión y exclusión de estatus_polizas
</commit_message>
<xml_diff>
--- a/legion_centurion/legion_centurion.xlsx
+++ b/legion_centurion/legion_centurion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/legion_centurion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6D5233-0EF9-EE4A-A37F-42940B0A44D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46EBBA23-4A4F-1B44-B6A9-5DAA79EFE298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{B49CA26D-17E4-1041-9F6C-DBD86CE9FF01}"/>
   </bookViews>
@@ -591,33 +591,33 @@
     </dxf>
     <dxf>
       <border>
-        <left style="hair">
-          <color indexed="64"/>
+        <left style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
         </left>
-        <right style="hair">
-          <color indexed="64"/>
+        <right style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
         </right>
-        <top style="hair">
-          <color indexed="64"/>
+        <top style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
         </top>
-        <bottom style="hair">
-          <color indexed="64"/>
+        <bottom style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
       <border>
-        <left style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
+        <left style="hair">
+          <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
+        <right style="hair">
+          <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
+        <top style="hair">
+          <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
+        <bottom style="hair">
+          <color indexed="64"/>
         </bottom>
       </border>
     </dxf>
@@ -1362,9 +1362,11 @@
     <sheetNames>
       <sheetName val="Respuestas de formulario 1"/>
       <sheetName val="Asesores"/>
-      <sheetName val="ESTATUS"/>
+      <sheetName val="ESTATUS AYER"/>
+      <sheetName val="ESTATUS HOY"/>
       <sheetName val="BD PROACTIVOS"/>
       <sheetName val="PROACTIVOS"/>
+      <sheetName val="Hoja2"/>
       <sheetName val="Ventas Mensuales"/>
       <sheetName val="EMIT &amp; PAG"/>
       <sheetName val="RANKING PROMOTORES"/>
@@ -1404,6 +1406,8 @@
       <sheetData sheetId="18"/>
       <sheetData sheetId="19"/>
       <sheetData sheetId="20"/>
+      <sheetData sheetId="21"/>
+      <sheetData sheetId="22"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1813,26 +1817,26 @@
         <v>46071</v>
       </c>
       <c r="D2" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" s="28">
         <v>4</v>
       </c>
       <c r="F2" s="3">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G2" s="15">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="H2" s="15">
-        <v>11</v>
+        <v>18.5</v>
       </c>
       <c r="I2" s="20">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="J2" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>2</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="K2" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -1852,26 +1856,26 @@
       </c>
       <c r="D3" s="1">
         <f>D2</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" s="28">
         <v>2.5</v>
       </c>
       <c r="F3" s="3">
-        <v>5.5</v>
+        <v>9.5</v>
       </c>
       <c r="G3" s="15">
-        <v>9.5</v>
+        <v>15.5</v>
       </c>
       <c r="H3" s="15">
-        <v>12.5</v>
+        <v>20</v>
       </c>
       <c r="I3" s="20">
-        <v>17.5</v>
+        <v>27.5</v>
       </c>
       <c r="J3" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>1.25</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="K3" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -1891,26 +1895,26 @@
       </c>
       <c r="D4" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" s="28">
         <v>1.5</v>
       </c>
       <c r="F4" s="3">
-        <v>6.5</v>
+        <v>10.5</v>
       </c>
       <c r="G4" s="15">
-        <v>10.5</v>
+        <v>16.5</v>
       </c>
       <c r="H4" s="15">
-        <v>13.5</v>
+        <v>21</v>
       </c>
       <c r="I4" s="20">
-        <v>18.5</v>
+        <v>28.5</v>
       </c>
       <c r="J4" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="K4" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -1930,26 +1934,26 @@
       </c>
       <c r="D5" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" s="28">
         <v>1.5</v>
       </c>
       <c r="F5" s="3">
-        <v>6.5</v>
+        <v>10.5</v>
       </c>
       <c r="G5" s="15">
-        <v>10.5</v>
+        <v>16.5</v>
       </c>
       <c r="H5" s="15">
-        <v>13.5</v>
+        <v>21</v>
       </c>
       <c r="I5" s="20">
-        <v>18.5</v>
+        <v>28.5</v>
       </c>
       <c r="J5" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="K5" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -1969,26 +1973,26 @@
       </c>
       <c r="D6" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" s="28">
         <v>1</v>
       </c>
       <c r="F6" s="3">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G6" s="15">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H6" s="15">
-        <v>14</v>
+        <v>21.5</v>
       </c>
       <c r="I6" s="20">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J6" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="K6" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2008,26 +2012,26 @@
       </c>
       <c r="D7" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" s="28">
         <v>1</v>
       </c>
       <c r="F7" s="3">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G7" s="15">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H7" s="15">
-        <v>14</v>
+        <v>21.5</v>
       </c>
       <c r="I7" s="20">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J7" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="K7" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2047,26 +2051,26 @@
       </c>
       <c r="D8" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E8" s="28">
         <v>1</v>
       </c>
       <c r="F8" s="3">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G8" s="15">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H8" s="15">
-        <v>14</v>
+        <v>21.5</v>
       </c>
       <c r="I8" s="20">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J8" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="K8" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2086,26 +2090,26 @@
       </c>
       <c r="D9" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" s="28">
         <v>1</v>
       </c>
       <c r="F9" s="3">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G9" s="15">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H9" s="15">
-        <v>14</v>
+        <v>21.5</v>
       </c>
       <c r="I9" s="20">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J9" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="K9" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2125,26 +2129,26 @@
       </c>
       <c r="D10" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" s="28">
         <v>1</v>
       </c>
       <c r="F10" s="3">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G10" s="15">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H10" s="15">
-        <v>14</v>
+        <v>21.5</v>
       </c>
       <c r="I10" s="20">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J10" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="K10" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2164,26 +2168,26 @@
       </c>
       <c r="D11" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" s="28">
         <v>1</v>
       </c>
       <c r="F11" s="3">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G11" s="15">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H11" s="15">
-        <v>14</v>
+        <v>21.5</v>
       </c>
       <c r="I11" s="20">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J11" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="K11" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2203,26 +2207,26 @@
       </c>
       <c r="D12" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" s="28">
         <v>1</v>
       </c>
       <c r="F12" s="3">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G12" s="15">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H12" s="15">
-        <v>14</v>
+        <v>21.5</v>
       </c>
       <c r="I12" s="20">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J12" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="K12" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2242,26 +2246,26 @@
       </c>
       <c r="D13" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E13" s="28">
         <v>1</v>
       </c>
       <c r="F13" s="3">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G13" s="15">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H13" s="15">
-        <v>14</v>
+        <v>21.5</v>
       </c>
       <c r="I13" s="20">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J13" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="K13" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2281,26 +2285,26 @@
       </c>
       <c r="D14" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E14" s="28">
         <v>1</v>
       </c>
       <c r="F14" s="3">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G14" s="15">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H14" s="15">
-        <v>14</v>
+        <v>21.5</v>
       </c>
       <c r="I14" s="20">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J14" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="K14" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2320,26 +2324,26 @@
       </c>
       <c r="D15" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" s="28">
         <v>0.5</v>
       </c>
       <c r="F15" s="3">
-        <v>7.5</v>
+        <v>11.5</v>
       </c>
       <c r="G15" s="15">
-        <v>11.5</v>
+        <v>17.5</v>
       </c>
       <c r="H15" s="15">
-        <v>14.5</v>
+        <v>22</v>
       </c>
       <c r="I15" s="20">
-        <v>19.5</v>
+        <v>29.5</v>
       </c>
       <c r="J15" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.25</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="K15" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2359,26 +2363,26 @@
       </c>
       <c r="D16" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E16" s="28">
         <v>0.5</v>
       </c>
       <c r="F16" s="3">
-        <v>7.5</v>
+        <v>11.5</v>
       </c>
       <c r="G16" s="15">
-        <v>11.5</v>
+        <v>17.5</v>
       </c>
       <c r="H16" s="15">
-        <v>14.5</v>
+        <v>22</v>
       </c>
       <c r="I16" s="20">
-        <v>19.5</v>
+        <v>29.5</v>
       </c>
       <c r="J16" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.25</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="K16" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2398,26 +2402,26 @@
       </c>
       <c r="D17" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E17" s="28">
         <v>0.5</v>
       </c>
       <c r="F17" s="3">
-        <v>7.5</v>
+        <v>11.5</v>
       </c>
       <c r="G17" s="15">
-        <v>11.5</v>
+        <v>17.5</v>
       </c>
       <c r="H17" s="15">
-        <v>14.5</v>
+        <v>22</v>
       </c>
       <c r="I17" s="20">
-        <v>19.5</v>
+        <v>29.5</v>
       </c>
       <c r="J17" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.25</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="K17" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2437,26 +2441,26 @@
       </c>
       <c r="D18" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E18" s="28">
         <v>0.5</v>
       </c>
       <c r="F18" s="3">
-        <v>7.5</v>
+        <v>11.5</v>
       </c>
       <c r="G18" s="15">
-        <v>11.5</v>
+        <v>17.5</v>
       </c>
       <c r="H18" s="15">
-        <v>14.5</v>
+        <v>22</v>
       </c>
       <c r="I18" s="20">
-        <v>19.5</v>
+        <v>29.5</v>
       </c>
       <c r="J18" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.25</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="K18" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2476,26 +2480,26 @@
       </c>
       <c r="D19" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E19" s="28">
         <v>0.5</v>
       </c>
       <c r="F19" s="3">
-        <v>7.5</v>
+        <v>11.5</v>
       </c>
       <c r="G19" s="15">
-        <v>11.5</v>
+        <v>17.5</v>
       </c>
       <c r="H19" s="15">
-        <v>14.5</v>
+        <v>22</v>
       </c>
       <c r="I19" s="20">
-        <v>19.5</v>
+        <v>29.5</v>
       </c>
       <c r="J19" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.25</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="K19" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2515,26 +2519,26 @@
       </c>
       <c r="D20" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E20" s="28">
         <v>0.5</v>
       </c>
       <c r="F20" s="3">
-        <v>7.5</v>
+        <v>11.5</v>
       </c>
       <c r="G20" s="15">
-        <v>11.5</v>
+        <v>17.5</v>
       </c>
       <c r="H20" s="15">
-        <v>14.5</v>
+        <v>22</v>
       </c>
       <c r="I20" s="20">
-        <v>19.5</v>
+        <v>29.5</v>
       </c>
       <c r="J20" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
-        <v>0.25</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="K20" s="25" t="str">
         <f>IF(Tabla1354[[#This Row],[Total_Polizas]] &gt;= (Tabla1354[[#This Row],[Mes_Actual]] * 4), "✅ EN META", "❌ POR DEBAJO")</f>
@@ -2554,22 +2558,22 @@
       </c>
       <c r="D21" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21" s="28">
         <v>0</v>
       </c>
       <c r="F21" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G21" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H21" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I21" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J21" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -2593,22 +2597,22 @@
       </c>
       <c r="D22" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E22" s="28">
         <v>0</v>
       </c>
       <c r="F22" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G22" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H22" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I22" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J22" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -2632,22 +2636,22 @@
       </c>
       <c r="D23" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E23" s="28">
         <v>0</v>
       </c>
       <c r="F23" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G23" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H23" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I23" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J23" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -2671,22 +2675,22 @@
       </c>
       <c r="D24" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E24" s="28">
         <v>0</v>
       </c>
       <c r="F24" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G24" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H24" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I24" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J24" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -2710,22 +2714,22 @@
       </c>
       <c r="D25" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E25" s="28">
         <v>0</v>
       </c>
       <c r="F25" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G25" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H25" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I25" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J25" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -2749,22 +2753,22 @@
       </c>
       <c r="D26" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E26" s="28">
         <v>0</v>
       </c>
       <c r="F26" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G26" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H26" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I26" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J26" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -2788,22 +2792,22 @@
       </c>
       <c r="D27" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E27" s="28">
         <v>0</v>
       </c>
       <c r="F27" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G27" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H27" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I27" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J27" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -2827,22 +2831,22 @@
       </c>
       <c r="D28" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28" s="28">
         <v>0</v>
       </c>
       <c r="F28" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G28" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H28" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I28" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J28" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -2866,22 +2870,22 @@
       </c>
       <c r="D29" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E29" s="28">
         <v>0</v>
       </c>
       <c r="F29" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G29" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H29" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I29" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J29" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -2905,22 +2909,22 @@
       </c>
       <c r="D30" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E30" s="28">
         <v>0</v>
       </c>
       <c r="F30" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G30" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H30" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I30" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J30" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -2944,22 +2948,22 @@
       </c>
       <c r="D31" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E31" s="28">
         <v>0</v>
       </c>
       <c r="F31" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G31" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H31" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I31" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J31" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -2983,22 +2987,22 @@
       </c>
       <c r="D32" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E32" s="28">
         <v>0</v>
       </c>
       <c r="F32" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G32" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H32" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I32" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J32" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3022,22 +3026,22 @@
       </c>
       <c r="D33" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E33" s="28">
         <v>0</v>
       </c>
       <c r="F33" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G33" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H33" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I33" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J33" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3061,22 +3065,22 @@
       </c>
       <c r="D34" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E34" s="28">
         <v>0</v>
       </c>
       <c r="F34" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G34" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H34" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I34" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J34" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3100,22 +3104,22 @@
       </c>
       <c r="D35" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E35" s="28">
         <v>0</v>
       </c>
       <c r="F35" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G35" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H35" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I35" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J35" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3139,22 +3143,22 @@
       </c>
       <c r="D36" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E36" s="28">
         <v>0</v>
       </c>
       <c r="F36" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G36" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H36" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I36" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J36" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3178,22 +3182,22 @@
       </c>
       <c r="D37" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E37" s="28">
         <v>0</v>
       </c>
       <c r="F37" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G37" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H37" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I37" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J37" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3217,22 +3221,22 @@
       </c>
       <c r="D38" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E38" s="28">
         <v>0</v>
       </c>
       <c r="F38" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G38" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H38" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I38" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J38" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3256,22 +3260,22 @@
       </c>
       <c r="D39" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E39" s="28">
         <v>0</v>
       </c>
       <c r="F39" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G39" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H39" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I39" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J39" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3295,22 +3299,22 @@
       </c>
       <c r="D40" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E40" s="28">
         <v>0</v>
       </c>
       <c r="F40" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G40" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H40" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I40" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J40" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3334,22 +3338,22 @@
       </c>
       <c r="D41" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E41" s="28">
         <v>0</v>
       </c>
       <c r="F41" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G41" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H41" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I41" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J41" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3373,22 +3377,22 @@
       </c>
       <c r="D42" s="1">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E42" s="28">
         <v>0</v>
       </c>
       <c r="F42" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G42" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H42" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I42" s="20">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J42" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3412,22 +3416,22 @@
       </c>
       <c r="D43" s="1">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E43" s="28">
         <v>0</v>
       </c>
       <c r="F43" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G43" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H43" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I43" s="21">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J43" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3451,22 +3455,22 @@
       </c>
       <c r="D44" s="1">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E44" s="28">
         <v>0</v>
       </c>
       <c r="F44" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G44" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H44" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I44" s="21">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J44" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3490,22 +3494,22 @@
       </c>
       <c r="D45" s="1">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E45" s="28">
         <v>0</v>
       </c>
       <c r="F45" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G45" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H45" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I45" s="21">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J45" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3529,22 +3533,22 @@
       </c>
       <c r="D46" s="1">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E46" s="28">
         <v>0</v>
       </c>
       <c r="F46" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G46" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H46" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I46" s="21">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J46" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3568,22 +3572,22 @@
       </c>
       <c r="D47" s="1">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E47" s="28">
         <v>0</v>
       </c>
       <c r="F47" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G47" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H47" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I47" s="21">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J47" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3607,22 +3611,22 @@
       </c>
       <c r="D48" s="1">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E48" s="28">
         <v>0</v>
       </c>
       <c r="F48" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G48" s="15">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H48" s="15">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="I48" s="21">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J48" s="23">
         <f>Tabla1354[[#This Row],[Total_Polizas]]/Tabla1354[[#This Row],[Mes_Actual]]</f>
@@ -3661,64 +3665,64 @@
     </row>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
-  <conditionalFormatting sqref="A3 C2:D49 G2:H49">
-    <cfRule type="expression" dxfId="14" priority="11" stopIfTrue="1">
-      <formula>#REF!&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A5">
-    <cfRule type="expression" dxfId="13" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="4" stopIfTrue="1">
       <formula>#REF!&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A7">
-    <cfRule type="expression" dxfId="12" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="9" stopIfTrue="1">
       <formula>#REF!&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A10">
-    <cfRule type="expression" dxfId="11" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="3" stopIfTrue="1">
       <formula>#REF!&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A12">
-    <cfRule type="expression" dxfId="10" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="7" stopIfTrue="1">
       <formula>#REF!&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A20">
-    <cfRule type="expression" dxfId="9" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="8" stopIfTrue="1">
       <formula>#REF!&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27">
-    <cfRule type="expression" dxfId="8" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="2" stopIfTrue="1">
       <formula>#REF!&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A35">
-    <cfRule type="expression" dxfId="7" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="5" stopIfTrue="1">
       <formula>#REF!&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A41">
-    <cfRule type="expression" dxfId="6" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="10" stopIfTrue="1">
       <formula>#REF!&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A45">
-    <cfRule type="expression" dxfId="5" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="6" stopIfTrue="1">
       <formula>#REF!&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A50:B50">
-    <cfRule type="expression" dxfId="4" priority="12" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="12" stopIfTrue="1">
       <formula>$B50&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B49">
-    <cfRule type="expression" dxfId="3" priority="14" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="14" stopIfTrue="1">
       <formula>$B49&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:D49 G2:H49 A3">
+    <cfRule type="expression" dxfId="3" priority="11" stopIfTrue="1">
+      <formula>#REF!&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E49">
@@ -3726,7 +3730,7 @@
       <formula>$B2&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E50:F50 F2:F49">
+  <conditionalFormatting sqref="F2:F49 E50:F50">
     <cfRule type="expression" dxfId="1" priority="16" stopIfTrue="1">
       <formula>#REF!&lt;&gt;""</formula>
     </cfRule>

</xml_diff>